<commit_message>
Add Jharkhand and West Bengal to the coverage matrix, fix a stale K-RERA row
RERA_Data_Coverage.xlsx only listed four authorities even though JHARERA and
WBRERA adapters have been live since Aug 20-21. Extend all 21 findings rows
to six states per what the adapters actually fetch, and correct K-RERA's
orders/judgments status from Partial to Yes now that all five of its
promoter-keyed order registers are wired up. Add three new rows to the
unused-findings sheet for JHARERA's unparsed balance sheet/ITR documents,
its unfetched rejected/surrendered lists, and WBRERA's unwired defaulters
parser.
</commit_message>
<xml_diff>
--- a/docs/RERA_Data_Coverage.xlsx
+++ b/docs/RERA_Data_Coverage.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D - Available but unused" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'A - RERA by authority'!$A$4:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'A - RERA by authority'!$A$4:$I$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'B - CTS land records'!$A$4:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'C - CIN corporate'!$A$4:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'D - Available but unused'!$A$4:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'D - Available but unused'!$A$4:$E$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -78,12 +78,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Regenerated 2026-08-19 by build_data_coverage.py</t>
+          <t>Regenerated 2026-08-21 by build_data_coverage.py</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>unaudited        nobody has looked. 26 of ~30 state portals are here.</t>
+          <t>unaudited        nobody has looked. 24 of ~30 state portals are here.</t>
         </is>
       </c>
     </row>
@@ -660,6 +660,20 @@
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>8. Group membership CANNOT be derived from a brand name. Searching 'PRANAMI' returns a Delhi hydro-power firm, a Gujarat non-profit and a Maharashtra castings company. Propose by name, confirm by shared director / registered office / filed relationship -- and treat a shared address as the weakest of the three (28 of 65 'group companies' were address-only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>9. Two more states are live: Jharkhand (JHARERA) and West Bengal (WBRERA), taking coverage to six authorities. JHARERA is the only authority anywhere in this pipeline that files a professional's PAN as a plain readable field rather than a scanned card, and it also publishes a declared past-projects table and a genuine litigation disclosure per project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>10. Karnataka's order/judgment coverage grew from one register to five (15,600+ rows across order search, authority orders, AO orders, interim orders and complaints-under-process), including a penalty table naming the violation, section and amount -- the single most consequential regulatory-history record any authority here publishes. JHARERA and WBRERA orders are now searchable by promoter too; WBRERA's join runs through its cause lists, since its own order register names no party directly.</t>
         </is>
       </c>
     </row>
@@ -674,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -682,8 +696,10 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -696,7 +712,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Yes / Partial / No / Not published / Unaudited. 'Unaudited' means nobody has looked yet -- 26 of ~30 state portals are in that state.</t>
+          <t>Yes / Partial / No / Not published / Unaudited. 'Unaudited' means nobody has looked yet -- 24 of ~30 state portals are in that state.</t>
         </is>
       </c>
     </row>
@@ -728,10 +744,20 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
+          <t>JHARERA</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>WBRERA</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
           <t>Charter facts field</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -763,12 +789,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>rera_core_fields</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr"/>
+      <c r="I5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -796,12 +832,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>rera_core_fields.registration_number</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>TG-RERA's public record does not display its own registration number; search is by project name.</t>
         </is>
@@ -833,12 +879,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>corporate_identity</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>K-RERA publishes partner PANs and land-owner SHARES -- neither appears on a MahaRERA record.</t>
         </is>
@@ -870,14 +926,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>local_planning.professionals_of_record</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>GujRERA splits these across englist/calist/acrchlist/contr; the adapter normalises to one list.</t>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>GujRERA splits these across englist/calist/acrchlist/contr; the adapter normalises to one list. JHARERA is the only authority here that files a professional's PAN as a plain text field -- for the contractor, architect and structural engineer -- rather than a scanned card.</t>
         </is>
       </c>
     </row>
@@ -907,14 +973,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>land_identification</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>K-RERA gives per-owner shares against survey numbers.</t>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>K-RERA gives per-owner shares against survey numbers. WBRERA's project page carries no land/survey table; not captured by this adapter, and whether the portal itself publishes one at all is unaudited.</t>
         </is>
       </c>
     </row>
@@ -944,14 +1020,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>rera_compliance.collection_account</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>TG-RERA publishes the 100% collection account but leaves the 70/30 split accounts blank.</t>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>TG-RERA publishes the 100% collection account but leaves the 70/30 split accounts blank. WBRERA's project page carries no bank-account table either -- same caveat as land details.</t>
         </is>
       </c>
     </row>
@@ -981,14 +1067,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>document_library</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>GujRERA 42/42 retrieved. K-RERA 112/152 -- the other 40 are LISTED but the portal serves 0 bytes.</t>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>GujRERA 42/42 retrieved. K-RERA 112/152 -- the other 40 are LISTED but the portal serves 0 bytes. JHARERA labels every document link 'View'; document_label() derives the real name from the surrounding table or header. WBRERA's links already carry real text, so no derivation is needed.</t>
         </is>
       </c>
     </row>
@@ -1018,14 +1114,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>rera_core_fields.total_complaints_count</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>K-RERA: use the STATE-WIDE /projectComplaintReport. The per-project page is NOT reliable -- it showed no complaints for a project the register lists with 12.</t>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>K-RERA: use the STATE-WIDE /projectComplaintReport. The per-project page is NOT reliable -- it showed no complaints for a project the register lists with 12. JHARERA has no per-project count either; the adapter name-matches the promoter against the state-wide disposed-complaint register, which yields POSSIBLE matches to confirm, not a confirmed count. WBRERA publishes no complaint register through this interface at all -- recorded as None, never 0.</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1161,22 @@
           <t>Not published</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>rera_core_fields.total_appeals_count</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1083,19 +1199,29 @@
           <t>Not published</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>sources[] (topic=litigation)</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>K-RERA /viewAllJudgements exists; the adapter reads complaints but not judgements yet.</t>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>K-RERA now reads FIVE promoter-keyed registers (order search, authority orders, AO orders, interim orders, complaints under process) -- 15,600+ rows including a penalty table naming the violation, section and amount. JHARERA's judgement/order register is searchable by promoter, though a share of rows name both parties in one unsplit column and are therefore invisible to that search. WBRERA's order register names no party at all; the join runs through its cause lists instead, so its coverage note matters more than its row count.</t>
         </is>
       </c>
     </row>
@@ -1125,14 +1251,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>promoter_portfolio</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>K-RERA embeds the WHOLE state index client-side (9,888 projects with promoter names), so a portfolio is one request. GujRERA confirmed absent.</t>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>K-RERA embeds the WHOLE state index client-side (9,888 projects with promoter names), so a portfolio is one request. GujRERA confirmed absent. WBRERA publishes no promoter search and its state index does not name the promoter either, so a portfolio there would mean opening all ~4,700 project pages -- the adapter returns None and says why rather than sampling a partial set.</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1298,22 @@
           <t>Not published</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>promoter_portfolio.totals</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr"/>
+      <c r="I16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1190,19 +1336,29 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>(unmapped -- see Charter Mapping sheet)</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>GujRERA findoc block. MahaRERA publishes nothing equivalent. Highest-value differential finding.</t>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>GujRERA findoc block. MahaRERA publishes nothing equivalent. Highest-value differential finding. JHARERA also files an audited balance sheet as a downloadable document, labelled directly on the project page.</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1388,22 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t>GujRERA findoc block.</t>
         </is>
@@ -1269,14 +1435,24 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>GujRERA findoc block.</t>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>GujRERA findoc block. JHARERA files three years of income-tax returns per project, also as downloadable documents.</t>
         </is>
       </c>
     </row>
@@ -1301,19 +1477,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>K-RERA /viewDefaultProjects -- observed, not yet built. No other authority publishes one.</t>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>K-RERA /viewDefaultProjects -- observed, not yet built. JHARERA's REJECTED and SURRENDERED registers are the closest equivalent: their URLs are imported into the adapter but nothing fetches them yet. WBRERA's defaulters list (17 rejected/defaulting applications by name) IS parsed by adapter_westbengal.fetch_defaulters(), but that function is called from nowhere in acquire() or the litigation sweep -- written, untested against a live page, and unused.</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1524,27 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>K-RERA /unregProjectList -- observed, not yet built.</t>
         </is>
@@ -1370,7 +1566,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1380,12 +1576,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>K-RERA publishes both, per particular. Direct input to the financial-strength sub-metric.</t>
         </is>
@@ -1417,12 +1623,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>K-RERA detail page carries a delay-reason table.</t>
         </is>
@@ -1454,12 +1670,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>(unmapped)</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>K-RERA tracks NOC validity dates and whether renewed.</t>
         </is>
@@ -1476,7 +1702,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1491,18 +1717,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Unaudited</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Unaudited</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>rera_compliance.construction_progress</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Not confirmed either way for JHARERA or WBRERA -- neither adapter currently extracts a QPR-equivalent field, and nobody has checked whether either portal even publishes one.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G25"/>
+  <autoFilter ref="A4:I25"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1582,7 +1822,7 @@
           <t>Maha Bhulekh Property Card (हक्काचा मूळ धारक)</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1614,7 +1854,7 @@
           <t>Maha Bhulekh Property Card (क्षेत्र चौ.मी.)</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1646,7 +1886,7 @@
           <t>Maha Bhulekh Property Card (धारणाधिकार)</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1678,7 +1918,7 @@
           <t>Maha Bhulekh Property Card (इतर भार)</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1710,7 +1950,7 @@
           <t>Maha Bhulekh Property Card (फेरफार table)</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1752,7 +1992,7 @@
           <t>Free + CAPTCHA</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>observed</t>
         </is>
@@ -1784,7 +2024,7 @@
           <t>Free + CAPTCHA</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>observed</t>
         </is>
@@ -1816,7 +2056,7 @@
           <t>Free -- page already fetched</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>observed</t>
         </is>
@@ -1838,7 +2078,7 @@
           <t>Dharani (TG) / Bhoomi (KA) / AnyROR (GJ) / Bhulekh (UP)</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Not built</t>
         </is>
@@ -1848,7 +2088,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>unaudited</t>
         </is>
@@ -2278,7 +2518,7 @@
           <t>ICRA / Infomerics press releases</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -2288,7 +2528,7 @@
           <t>Free</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>observed</t>
         </is>
@@ -2320,7 +2560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2473,7 +2713,7 @@
           <t>Same -- a regulator-declared adverse signal.</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2500,7 +2740,7 @@
           <t>Free route to revenue/debt/net-worth figures the MCA charges for.</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2554,7 +2794,7 @@
           <t>Promoter-declared delay reasons and lapsed-NOC tracking; no equivalent elsewhere.</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2587,8 +2827,89 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>JHARERA audited balance sheet + 3 years ITR</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>adapter_jharkhand.py document library (labelled, downloaded)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Jharkhand projects</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Same gap as GujRERA's findoc block: the financial-strength sub-metric scores None for every project regardless of state. This would score it for JH too.</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>JHARERA rejected + surrendered registration lists</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>REJECTED_LIST / SURRENDERED_LIST, imported into the adapter but never fetched</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Jharkhand projects</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>A rejected or surrendered registration is diligence material with no equivalent on MahaRERA. The URLs are already wired into the import list; nothing calls them yet.</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>WBRERA defaulters list</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>adapter_westbengal.fetch_defaulters() -- written, unwired, untested live</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>West Bengal projects</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>17 rejected/defaulting applications keyed by name -- a cheap, direct red-flag input. The parser exists but is called from nowhere in acquire() or the litigation sweep.</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E12"/>
+  <autoFilter ref="A4:E15"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
Reconcile a stale CTS row against the already-confirmed CIN one
Sheet B's "Lender, amount, satisfaction status" row still said
observed/"NOT currently parsed" for the MCA charge filings, months
after Sheet C's own row for the same underlying fact (company_
profile_check.charges) was confirmed live in commit d0536e6 -- this
one just never got updated to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/RERA_Data_Coverage.xlsx
+++ b/docs/RERA_Data_Coverage.xlsx
@@ -2546,14 +2546,14 @@
           <t>Free -- page already fetched</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>observed</t>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>confirmed-live</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>NOT currently parsed. The only independent check on the promoter's declared mortgage. National, so it belongs in the CIN workflow.</t>
+          <t>STALE ROW, RECONCILED 2026-09-01: this said 'observed'/'NOT currently parsed' months after it actually was -- company_profile_check.charges was wired up and confirmed live on 2026-08-19 (commit d0536e6), and Sheet C's own 'MCA CHARGE FILINGS' row has said confirmed-live since then. This row just never got updated to match. See that row for the live evidence (4 open charges, ~Rs 90.3 crore, HDFC Bank and Catalyst Trusteeship) -- kept here too, duplicated rather than deleted, because this is the only independent check on a promoter's declared mortgage and a reader scanning the land-records sheet for that fact should not be told it is still unbuilt.</t>
         </is>
       </c>
     </row>

</xml_diff>